<commit_message>
feat: enhance main functionality with screenshot and Excel generation features fix: improve Chrome driver options for better performance chore: update requirements.txt with additional dependencies
</commit_message>
<xml_diff>
--- a/trackcoder.xlsx
+++ b/trackcoder.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,6 +550,48 @@
       </c>
       <c r="J3" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-10-30</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7:55</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>6:00</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>